<commit_message>
directory: add Justice Hayes + Octavious (hired 2026-09-24, phones pending)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Justice</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kaisha</t>
+          <t>Kable</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 439-9802</t>
+          <t>(502) 606-3088</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Kasey</t>
+          <t>Kaisha</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 884-2273</t>
+          <t>(502) 439-9802</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -780,12 +780,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Kasey</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>(502) 531-8704</t>
+          <t>(502) 884-2273</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Kenzie</t>
+          <t>Kayla</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>(502) 650-2273</t>
+          <t>(502) 531-8704</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Lidy</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(502) 381-0680</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Madelynn</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(502) 938-3999</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -848,12 +848,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Maylin</t>
+          <t>Madelynn</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(502) 803-1973</t>
+          <t>(502) 938-3999</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Megan</t>
+          <t>Maylin</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(502) 833-2695</t>
+          <t>(502) 803-1973</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -882,12 +882,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Megan</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>(502) 281-8177</t>
+          <t>(502) 833-2695</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Mike</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>(502) 693-8371</t>
+          <t>(502) 281-8177</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -916,12 +916,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Nyatiek</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>(502) 576-1634</t>
+          <t>(502) 693-8371</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -933,12 +933,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Richard Gibbs</t>
+          <t>Nyatiek</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>(270) 874-0688</t>
+          <t>(502) 576-1634</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -950,12 +950,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Rusul</t>
+          <t>Richard Gibbs</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>(502) 656-9660</t>
+          <t>(270) 874-0688</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -967,12 +967,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vititoe</t>
+          <t>Octavious</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>(502) 528-7789</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -984,12 +984,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>(502) 724-2384</t>
+          <t>(502) 656-9660</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1001,12 +1001,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Serina</t>
+          <t>Ryan Vititoe</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>(502) 777-7987</t>
+          <t>(502) 528-7789</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1018,12 +1018,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(502) 724-2384</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1035,22 +1035,56 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>Serina</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>(502) 777-7987</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C35"/>
+  <autoFilter ref="A1:C37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
directory: sync to Teamworx schedule WE 9/27 — 18 active (15 scheduled + Justice Hayes, Octavious Cambron, Jeanie)
Removed 23 crew not on the schedule. Added scheduled crew missing from directory:
Elizabeth, Emanuela, Madison, Robert Muncy. Phones for Justice + Octavious from Bobby.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Angela</t>
+          <t>Anthony</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>(502) 912-4944</t>
+          <t>(502) 938-5182</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -508,12 +508,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Anthony</t>
+          <t>Cortez</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>(502) 938-5182</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -525,12 +525,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Ash</t>
+          <t>Elizabeth</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>(502) 554-4833</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -542,12 +542,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>Emanuela</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>(502) 656-2133</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -559,12 +559,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Bri</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>(502) 202-4126</t>
+          <t>(407) 456-1445</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -576,12 +576,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Chloe</t>
+          <t>Javeh</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(502) 382-5315</t>
+          <t>(502) 216-4460</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cortez</t>
+          <t>Jeanie</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dakayla</t>
+          <t>Justice</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>(502) 537-8724</t>
+          <t>(502) 936-5610</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -627,12 +627,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Divan</t>
+          <t>Kenzie</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-9406</t>
+          <t>(502) 650-2273</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Lidy</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>(407) 456-1445</t>
+          <t>(502) 381-0680</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Madelynn</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>(502) 527-1477</t>
+          <t>(502) 938-3999</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -678,12 +678,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Jada</t>
+          <t>Madison</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(502) 821-5962</t>
+          <t>(502) 938-9208</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Javeh</t>
+          <t>Octavious</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(502) 216-4460</t>
+          <t>(502) 649-6790</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -712,12 +712,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Robert Muncy</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(502) 498-9401</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Justice</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(PHONE PENDING)</t>
+          <t>(502) 656-9660</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kable</t>
+          <t>Vicki</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 606-3088</t>
+          <t>(502) 701-9597</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Kaisha</t>
+          <t>Zach</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(502) 439-9802</t>
+          <t>(502) 422-9066</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -777,314 +777,8 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Kasey</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>(502) 884-2273</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Kayla</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>(502) 531-8704</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Kenzie</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>(502) 650-2273</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Lidy</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>(502) 381-0680</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Madelynn</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>(502) 938-3999</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Maylin</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>(502) 803-1973</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Megan</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>(502) 833-2695</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Mike</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>(502) 281-8177</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Nathan</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>(502) 693-8371</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Nyatiek</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>(502) 576-1634</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Richard Gibbs</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>(270) 874-0688</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Octavious</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>(PHONE PENDING)</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Rusul</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>(502) 656-9660</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Ryan Vititoe</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>(502) 528-7789</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Samuel</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>(502) 724-2384</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Serina</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>(502) 777-7987</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Vicki</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>(502) 701-9597</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Zach</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>(502) 422-9066</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C37"/>
+  <autoFilter ref="A1:C19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
directory: add Rodolfo (new hire 2026-10-22, phone pending)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/employee_directory.xlsx
+++ b/employee_directory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Employees'!$A$1:$C$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -729,12 +729,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Rusul</t>
+          <t>Rodolfo</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>(502) 656-9660</t>
+          <t>(PHONE PENDING)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Vicki</t>
+          <t>Rusul</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(502) 701-9597</t>
+          <t>(502) 656-9660</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -763,22 +763,39 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>(502) 701-9597</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Zach</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>(502) 422-9066</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C19"/>
+  <autoFilter ref="A1:C20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>